<commit_message>
Update on script stabilization
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/CreditCardDetailViewData.xlsx
+++ b/src/test/resources/TEST_DATA/CreditCardDetailViewData.xlsx
@@ -33,7 +33,7 @@
     <t>100</t>
   </si>
   <si>
-    <t xml:space="preserve">Request successful</t>
+    <t xml:space="preserve">Payment Complete</t>
   </si>
 </sst>
 </file>
@@ -578,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" style="1" width="35.8515625"/>
     <col customWidth="1" min="2" max="2" style="1" width="81.8515625"/>
@@ -587,13 +587,13 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -601,7 +601,7 @@
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="2" t="s">

</xml_diff>

<commit_message>
commit the changes that done to CreditCarddetailedView,LoanAccountDetail,ObtainLoan,Pawning pages with test and data files
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/CreditCardDetailViewData.xlsx
+++ b/src/test/resources/TEST_DATA/CreditCardDetailViewData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>payingAccountNumber</t>
   </si>
@@ -24,6 +24,9 @@
     <t>paymentAmount</t>
   </si>
   <si>
+    <t>errorMsg</t>
+  </si>
+  <si>
     <t>successMsg</t>
   </si>
   <si>
@@ -31,6 +34,9 @@
   </si>
   <si>
     <t>100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custom amount must be greater than 0</t>
   </si>
   <si>
     <t xml:space="preserve">Request successful</t>
@@ -578,34 +584,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" style="1" width="35.8515625"/>
-    <col customWidth="1" min="2" max="2" style="1" width="81.8515625"/>
-    <col customWidth="1" min="3" max="3" style="1" width="39.8515625"/>
-    <col min="4" max="16384" style="1" width="9.140625"/>
+    <col customWidth="1" min="2" max="3" style="1" width="81.8515625"/>
+    <col customWidth="1" min="4" max="4" style="1" width="39.8515625"/>
+    <col min="5" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
commit the changes of the credit card data sheet
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/CreditCardDetailViewData.xlsx
+++ b/src/test/resources/TEST_DATA/CreditCardDetailViewData.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>payingAccountNumber</t>
   </si>
@@ -27,6 +27,9 @@
     <t>successMsg</t>
   </si>
   <si>
+    <t>errorMsg</t>
+  </si>
+  <si>
     <t>112653780142</t>
   </si>
   <si>
@@ -34,6 +37,9 @@
   </si>
   <si>
     <t xml:space="preserve">Payment Complete</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custom amount must be greater than 0</t>
   </si>
 </sst>
 </file>
@@ -596,16 +602,22 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
+      <c r="A2" s="1" t="s">
+        <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
         <v>5</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
commit the updates and stabilization done to CreditCardDetailedViewPage.java,DashBoardPage,LoanAccoutdetailPage,OpenFD,OpenSavings,Pawning.and data sheets settings,SavingsandFDdata,Creditcard,LoanDetails
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/CreditCardDetailViewData.xlsx
+++ b/src/test/resources/TEST_DATA/CreditCardDetailViewData.xlsx
@@ -16,11 +16,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>payingAccountNumber</t>
   </si>
   <si>
+    <t>ZeroAmount</t>
+  </si>
+  <si>
     <t>paymentAmount</t>
   </si>
   <si>
@@ -30,9 +33,21 @@
     <t>errorMsg</t>
   </si>
   <si>
+    <t>successMsgForBlocking</t>
+  </si>
+  <si>
+    <t>emailSentSuccessMsg</t>
+  </si>
+  <si>
+    <t>InsufficientamountErr</t>
+  </si>
+  <si>
     <t>112653780142</t>
   </si>
   <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>100</t>
   </si>
   <si>
@@ -40,6 +55,15 @@
   </si>
   <si>
     <t xml:space="preserve">Custom amount must be greater than 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request successful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMS sent successfully to the registered mobile number:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insufficient funds in the selected account</t>
   </si>
 </sst>
 </file>
@@ -586,10 +610,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="1" width="35.8515625"/>
-    <col customWidth="1" min="2" max="2" style="1" width="81.8515625"/>
-    <col customWidth="1" min="3" max="3" style="1" width="39.8515625"/>
-    <col min="4" max="16384" style="1" width="9.140625"/>
+    <col customWidth="1" min="1" max="2" style="1" width="35.8515625"/>
+    <col customWidth="1" min="3" max="3" style="1" width="81.8515625"/>
+    <col customWidth="1" min="4" max="4" style="1" width="39.8515625"/>
+    <col customWidth="1" min="5" max="5" style="1" width="37.00390625"/>
+    <col customWidth="1" min="6" max="6" style="1" width="27.7109375"/>
+    <col customWidth="1" min="7" max="7" style="1" width="35.140625"/>
+    <col customWidth="1" min="8" max="8" style="1" width="26.57421875"/>
+    <col min="9" max="16384" style="1" width="9.140625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -602,22 +630,46 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
-        <v>4</v>
+      <c r="A2" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
+        <v>10</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>